<commit_message>
pulse experiments for SI3
</commit_message>
<xml_diff>
--- a/experiments/pulse_experiments/pulse_experiment_hydrographs.xlsx
+++ b/experiments/pulse_experiments/pulse_experiment_hydrographs.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nicol\Documents\GitHub\La_Jara\Hysteresis\Experiments-Summer2022\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\huck4481\Documents\GitHub\hysteresis\experiments\pulse_experiments\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6FD96B1-A77E-4531-86A6-7830A4DB50D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{064D206E-3822-4F71-86EF-5770943440BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{055D4222-03BB-4B33-97D6-42AEC377BEC2}"/>
+    <workbookView xWindow="-25320" yWindow="360" windowWidth="25440" windowHeight="15270" xr2:uid="{055D4222-03BB-4B33-97D6-42AEC377BEC2}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="for SI" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="26">
   <si>
     <t>Time</t>
   </si>
@@ -73,12 +74,57 @@
   <si>
     <t>EXP 8</t>
   </si>
+  <si>
+    <t>Experiment 2</t>
+  </si>
+  <si>
+    <t>Experiment 3</t>
+  </si>
+  <si>
+    <t>Experiment 4</t>
+  </si>
+  <si>
+    <t>Experiment 5</t>
+  </si>
+  <si>
+    <t>Experiment 6</t>
+  </si>
+  <si>
+    <t>Experiment 7</t>
+  </si>
+  <si>
+    <t>Experiment 8</t>
+  </si>
+  <si>
+    <t>PP (mg/L)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Experiment </t>
+  </si>
+  <si>
+    <t>SS (mg/L)</t>
+  </si>
+  <si>
+    <t>POC (mg/L)</t>
+  </si>
+  <si>
+    <t>DOC (mg/L)</t>
+  </si>
+  <si>
+    <t>SRP (mg/L)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Time </t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.000"/>
+  </numFmts>
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -86,16 +132,58 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-9.9978637043366805E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -103,11 +191,26 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -116,6 +219,72 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="21" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="21" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="21" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="21" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -456,7 +625,7 @@
             <c:numRef>
               <c:f>Sheet1!$C$3:$C$16</c:f>
               <c:numCache>
-                <c:formatCode>General</c:formatCode>
+                <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="14"/>
                 <c:pt idx="0">
                   <c:v>9.2750000000000004</c:v>
@@ -742,7 +911,7 @@
             </a:p>
           </c:txPr>
         </c:title>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="0.00" sourceLinked="1"/>
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -795,6 +964,7 @@
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:crossAx val="37644799"/>
+        <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:spPr>
@@ -838,6 +1008,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -845,7 +1016,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -1160,7 +1330,7 @@
             <c:numRef>
               <c:f>Sheet1!$AM$3:$AM$15</c:f>
               <c:numCache>
-                <c:formatCode>General</c:formatCode>
+                <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="13"/>
                 <c:pt idx="0">
                   <c:v>7.2329999999999997</c:v>
@@ -1437,7 +1607,7 @@
             </a:p>
           </c:txPr>
         </c:title>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="0.00" sourceLinked="1"/>
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -1534,6 +1704,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -1541,7 +1712,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -1870,7 +2040,7 @@
             <c:numRef>
               <c:f>Sheet1!$U$3:$U$18</c:f>
               <c:numCache>
-                <c:formatCode>General</c:formatCode>
+                <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="16"/>
                 <c:pt idx="0">
                   <c:v>5.3079999999999998</c:v>
@@ -2150,7 +2320,7 @@
             </a:p>
           </c:txPr>
         </c:title>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="0.00" sourceLinked="1"/>
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -2247,6 +2417,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -2254,7 +2425,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -2592,7 +2762,7 @@
             <c:numRef>
               <c:f>Sheet1!$AA$3:$AA$18</c:f>
               <c:numCache>
-                <c:formatCode>General</c:formatCode>
+                <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="16"/>
                 <c:pt idx="0">
                   <c:v>3.5579999999999998</c:v>
@@ -2875,7 +3045,7 @@
             </a:p>
           </c:txPr>
         </c:title>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="0.00" sourceLinked="1"/>
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -2972,6 +3142,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -2979,7 +3150,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -3299,7 +3469,7 @@
             <c:numRef>
               <c:f>Sheet1!$AG$3:$AG$18</c:f>
               <c:numCache>
-                <c:formatCode>General</c:formatCode>
+                <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="16"/>
                 <c:pt idx="0">
                   <c:v>8.4580000000000002</c:v>
@@ -3578,7 +3748,7 @@
             </a:p>
           </c:txPr>
         </c:title>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="0.00" sourceLinked="1"/>
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -3675,6 +3845,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -3682,7 +3853,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -4008,7 +4178,7 @@
             <c:numRef>
               <c:f>Sheet1!$AM$3:$AM$13</c:f>
               <c:numCache>
-                <c:formatCode>General</c:formatCode>
+                <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="11"/>
                 <c:pt idx="0">
                   <c:v>7.2329999999999997</c:v>
@@ -4287,7 +4457,7 @@
             </a:p>
           </c:txPr>
         </c:title>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="0.00" sourceLinked="1"/>
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -4384,6 +4554,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -4391,7 +4562,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -4739,7 +4909,7 @@
             <c:numRef>
               <c:f>Sheet1!$C$3:$C$16</c:f>
               <c:numCache>
-                <c:formatCode>General</c:formatCode>
+                <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="14"/>
                 <c:pt idx="0">
                   <c:v>9.2750000000000004</c:v>
@@ -5025,7 +5195,7 @@
             </a:p>
           </c:txPr>
         </c:title>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="0.00" sourceLinked="1"/>
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -5122,6 +5292,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -5129,7 +5300,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -5495,7 +5665,7 @@
             <c:numRef>
               <c:f>Sheet1!$I$3:$I$18</c:f>
               <c:numCache>
-                <c:formatCode>General</c:formatCode>
+                <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="16"/>
                 <c:pt idx="0">
                   <c:v>10.092000000000001</c:v>
@@ -5787,7 +5957,7 @@
             </a:p>
           </c:txPr>
         </c:title>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="0.00" sourceLinked="1"/>
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -5884,6 +6054,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -5891,7 +6062,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -6230,7 +6400,7 @@
             <c:numRef>
               <c:f>Sheet1!$O$3:$O$15</c:f>
               <c:numCache>
-                <c:formatCode>General</c:formatCode>
+                <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="13"/>
                 <c:pt idx="0">
                   <c:v>8.3420000000000005</c:v>
@@ -6513,7 +6683,7 @@
             </a:p>
           </c:txPr>
         </c:title>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="0.00" sourceLinked="1"/>
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -6610,6 +6780,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -6617,7 +6788,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -6982,7 +7152,7 @@
             <c:numRef>
               <c:f>Sheet1!$I$3:$I$18</c:f>
               <c:numCache>
-                <c:formatCode>General</c:formatCode>
+                <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="16"/>
                 <c:pt idx="0">
                   <c:v>10.092000000000001</c:v>
@@ -7274,7 +7444,7 @@
             </a:p>
           </c:txPr>
         </c:title>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="0.00" sourceLinked="1"/>
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -7371,6 +7541,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -7378,7 +7549,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -7716,7 +7886,7 @@
             <c:numRef>
               <c:f>Sheet1!$O$3:$O$18</c:f>
               <c:numCache>
-                <c:formatCode>General</c:formatCode>
+                <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="16"/>
                 <c:pt idx="0">
                   <c:v>8.3420000000000005</c:v>
@@ -7999,7 +8169,7 @@
             </a:p>
           </c:txPr>
         </c:title>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="0.00" sourceLinked="1"/>
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -8096,6 +8266,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -8103,7 +8274,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -8427,7 +8597,7 @@
             <c:numRef>
               <c:f>Sheet1!$U$3:$U$15</c:f>
               <c:numCache>
-                <c:formatCode>General</c:formatCode>
+                <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="13"/>
                 <c:pt idx="0">
                   <c:v>5.3079999999999998</c:v>
@@ -8707,7 +8877,7 @@
             </a:p>
           </c:txPr>
         </c:title>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="0.00" sourceLinked="1"/>
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -8804,6 +8974,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -8811,7 +8982,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -9144,7 +9314,7 @@
             <c:numRef>
               <c:f>Sheet1!$AA$3:$AA$15</c:f>
               <c:numCache>
-                <c:formatCode>General</c:formatCode>
+                <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="13"/>
                 <c:pt idx="0">
                   <c:v>3.5579999999999998</c:v>
@@ -9427,7 +9597,7 @@
             </a:p>
           </c:txPr>
         </c:title>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="0.00" sourceLinked="1"/>
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -9524,6 +9694,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -9531,7 +9702,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -9837,7 +10007,7 @@
             <c:numRef>
               <c:f>Sheet1!$AG$4:$AG$15</c:f>
               <c:numCache>
-                <c:formatCode>General</c:formatCode>
+                <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="12"/>
                 <c:pt idx="0">
                   <c:v>8.6329999999999991</c:v>
@@ -10111,7 +10281,7 @@
             </a:p>
           </c:txPr>
         </c:title>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="0.00" sourceLinked="1"/>
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -10208,6 +10378,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -10215,7 +10386,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -18549,9 +18719,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -18589,7 +18759,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -18695,7 +18865,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -18837,7 +19007,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -19017,7 +19187,7 @@
       <c r="B3" s="2">
         <v>0.49802083333333336</v>
       </c>
-      <c r="C3" s="1">
+      <c r="C3" s="27">
         <v>9.2750000000000004</v>
       </c>
       <c r="D3" s="1">
@@ -19032,7 +19202,7 @@
       <c r="H3" s="2">
         <v>7.8923611111111111E-2</v>
       </c>
-      <c r="I3" s="1">
+      <c r="I3" s="27">
         <v>10.092000000000001</v>
       </c>
       <c r="J3" s="1">
@@ -19047,7 +19217,7 @@
       <c r="N3" s="2">
         <v>0.10474537037037036</v>
       </c>
-      <c r="O3" s="1">
+      <c r="O3" s="27">
         <v>8.3420000000000005</v>
       </c>
       <c r="P3" s="1">
@@ -19062,7 +19232,7 @@
       <c r="T3" s="2">
         <v>0.4397685185185185</v>
       </c>
-      <c r="U3" s="1">
+      <c r="U3" s="27">
         <v>5.3079999999999998</v>
       </c>
       <c r="V3" s="1">
@@ -19077,7 +19247,7 @@
       <c r="Z3" s="2">
         <v>0.46828703703703706</v>
       </c>
-      <c r="AA3" s="1">
+      <c r="AA3" s="27">
         <v>3.5579999999999998</v>
       </c>
       <c r="AB3" s="1">
@@ -19092,7 +19262,7 @@
       <c r="AF3" s="2">
         <v>8.261574074074074E-2</v>
       </c>
-      <c r="AG3" s="1">
+      <c r="AG3" s="27">
         <v>8.4580000000000002</v>
       </c>
       <c r="AH3" s="1">
@@ -19107,7 +19277,7 @@
       <c r="AL3" s="2">
         <v>0.46894675925925927</v>
       </c>
-      <c r="AM3" s="1">
+      <c r="AM3" s="27">
         <v>7.2329999999999997</v>
       </c>
       <c r="AN3" s="1">
@@ -19124,7 +19294,7 @@
       <c r="B4" s="2">
         <v>0.49815972222222221</v>
       </c>
-      <c r="C4" s="1">
+      <c r="C4" s="27">
         <v>22.75</v>
       </c>
       <c r="D4" s="1">
@@ -19139,7 +19309,7 @@
       <c r="H4" s="2">
         <v>7.9050925925925927E-2</v>
       </c>
-      <c r="I4" s="1">
+      <c r="I4" s="27">
         <v>10.382999999999999</v>
       </c>
       <c r="J4" s="1">
@@ -19154,7 +19324,7 @@
       <c r="N4" s="2">
         <v>0.10486111111111111</v>
       </c>
-      <c r="O4" s="1">
+      <c r="O4" s="27">
         <v>21.641999999999999</v>
       </c>
       <c r="P4" s="1">
@@ -19169,7 +19339,7 @@
       <c r="T4" s="2">
         <v>0.44150462962962966</v>
       </c>
-      <c r="U4" s="1">
+      <c r="U4" s="27">
         <v>13.532999999999999</v>
       </c>
       <c r="V4" s="1">
@@ -19184,7 +19354,7 @@
       <c r="Z4" s="2">
         <v>0.47123842592592591</v>
       </c>
-      <c r="AA4" s="1">
+      <c r="AA4" s="27">
         <v>7.5250000000000004</v>
       </c>
       <c r="AB4" s="1">
@@ -19199,7 +19369,7 @@
       <c r="AF4" s="2">
         <v>8.396990740740741E-2</v>
       </c>
-      <c r="AG4" s="1">
+      <c r="AG4" s="27">
         <v>8.6329999999999991</v>
       </c>
       <c r="AH4" s="1">
@@ -19214,7 +19384,7 @@
       <c r="AL4" s="2">
         <v>0.4689814814814815</v>
       </c>
-      <c r="AM4" s="1">
+      <c r="AM4" s="27">
         <v>7.2329999999999997</v>
       </c>
       <c r="AN4" s="1">
@@ -19231,7 +19401,7 @@
       <c r="B5" s="2">
         <v>0.49828703703703708</v>
       </c>
-      <c r="C5" s="1">
+      <c r="C5" s="27">
         <v>19.25</v>
       </c>
       <c r="D5" s="1">
@@ -19246,7 +19416,7 @@
       <c r="H5" s="2">
         <v>7.9166666666666663E-2</v>
       </c>
-      <c r="I5" s="1">
+      <c r="I5" s="27">
         <v>21.992000000000001</v>
       </c>
       <c r="J5" s="1">
@@ -19261,7 +19431,7 @@
       <c r="N5" s="2">
         <v>0.10497685185185185</v>
       </c>
-      <c r="O5" s="1">
+      <c r="O5" s="27">
         <v>16.917000000000002</v>
       </c>
       <c r="P5" s="1">
@@ -19276,7 +19446,7 @@
       <c r="T5" s="2">
         <v>0.44156250000000002</v>
       </c>
-      <c r="U5" s="1">
+      <c r="U5" s="27">
         <v>14.816000000000001</v>
       </c>
       <c r="V5" s="1">
@@ -19291,7 +19461,7 @@
       <c r="Z5" s="2">
         <v>0.47129629629629632</v>
       </c>
-      <c r="AA5" s="1">
+      <c r="AA5" s="27">
         <v>12.132999999999999</v>
       </c>
       <c r="AB5" s="1">
@@ -19306,7 +19476,7 @@
       <c r="AF5" s="2">
         <v>8.4004629629629624E-2</v>
       </c>
-      <c r="AG5" s="1">
+      <c r="AG5" s="27">
         <v>8.8079999999999998</v>
       </c>
       <c r="AH5" s="1">
@@ -19321,7 +19491,7 @@
       <c r="AL5" s="2">
         <v>0.46901620370370373</v>
       </c>
-      <c r="AM5" s="1">
+      <c r="AM5" s="27">
         <v>7.9329999999999998</v>
       </c>
       <c r="AN5" s="1">
@@ -19338,7 +19508,7 @@
       <c r="B6" s="2">
         <v>0.49840277777777775</v>
       </c>
-      <c r="C6" s="1">
+      <c r="C6" s="27">
         <v>16.100000000000001</v>
       </c>
       <c r="D6" s="1">
@@ -19353,7 +19523,7 @@
       <c r="H6" s="2">
         <v>7.9282407407407399E-2</v>
       </c>
-      <c r="I6" s="1">
+      <c r="I6" s="27">
         <v>18.317</v>
       </c>
       <c r="J6" s="1">
@@ -19368,7 +19538,7 @@
       <c r="N6" s="2">
         <v>0.10509259259259258</v>
       </c>
-      <c r="O6" s="1">
+      <c r="O6" s="27">
         <v>14.175000000000001</v>
       </c>
       <c r="P6" s="1">
@@ -19383,7 +19553,7 @@
       <c r="T6" s="2">
         <v>0.44162037037037033</v>
       </c>
-      <c r="U6" s="1">
+      <c r="U6" s="27">
         <v>21.291</v>
       </c>
       <c r="V6" s="1">
@@ -19398,7 +19568,7 @@
       <c r="Z6" s="2">
         <v>0.47135416666666669</v>
       </c>
-      <c r="AA6" s="1">
+      <c r="AA6" s="27">
         <v>21.991</v>
       </c>
       <c r="AB6" s="1">
@@ -19413,7 +19583,7 @@
       <c r="AF6" s="2">
         <v>8.4039351851851851E-2</v>
       </c>
-      <c r="AG6" s="1">
+      <c r="AG6" s="27">
         <v>9.0419999999999998</v>
       </c>
       <c r="AH6" s="1">
@@ -19428,7 +19598,7 @@
       <c r="AL6" s="2">
         <v>0.4690509259259259</v>
       </c>
-      <c r="AM6" s="1">
+      <c r="AM6" s="27">
         <v>9.3919999999999995</v>
       </c>
       <c r="AN6" s="1">
@@ -19445,7 +19615,7 @@
       <c r="B7" s="2">
         <v>0.49853009259259262</v>
       </c>
-      <c r="C7" s="1">
+      <c r="C7" s="27">
         <v>13.884</v>
       </c>
       <c r="D7" s="1">
@@ -19460,7 +19630,7 @@
       <c r="H7" s="2">
         <v>7.9398148148148148E-2</v>
       </c>
-      <c r="I7" s="1">
+      <c r="I7" s="27">
         <v>15.983000000000001</v>
       </c>
       <c r="J7" s="1">
@@ -19475,7 +19645,7 @@
       <c r="N7" s="2">
         <v>0.10520833333333333</v>
       </c>
-      <c r="O7" s="1">
+      <c r="O7" s="27">
         <v>12.95</v>
       </c>
       <c r="P7" s="1">
@@ -19490,7 +19660,7 @@
       <c r="T7" s="2">
         <v>0.44167824074074075</v>
       </c>
-      <c r="U7" s="1">
+      <c r="U7" s="27">
         <v>18.140999999999998</v>
       </c>
       <c r="V7" s="1">
@@ -19505,7 +19675,7 @@
       <c r="Z7" s="2">
         <v>0.47141203703703699</v>
       </c>
-      <c r="AA7" s="1">
+      <c r="AA7" s="27">
         <v>23.274999999999999</v>
       </c>
       <c r="AB7" s="1">
@@ -19520,7 +19690,7 @@
       <c r="AF7" s="2">
         <v>8.4074074074074079E-2</v>
       </c>
-      <c r="AG7" s="1">
+      <c r="AG7" s="27">
         <v>9.9169999999999998</v>
       </c>
       <c r="AH7" s="1">
@@ -19535,7 +19705,7 @@
       <c r="AL7" s="2">
         <v>0.46908564814814818</v>
       </c>
-      <c r="AM7" s="1">
+      <c r="AM7" s="27">
         <v>9.3919999999999995</v>
       </c>
       <c r="AN7" s="1">
@@ -19552,7 +19722,7 @@
       <c r="B8" s="2">
         <v>0.49865740740740744</v>
       </c>
-      <c r="C8" s="1">
+      <c r="C8" s="27">
         <v>12.775</v>
       </c>
       <c r="D8" s="1">
@@ -19567,7 +19737,7 @@
       <c r="H8" s="2">
         <v>7.9513888888888884E-2</v>
       </c>
-      <c r="I8" s="1">
+      <c r="I8" s="27">
         <v>14.525</v>
       </c>
       <c r="J8" s="1">
@@ -19582,7 +19752,7 @@
       <c r="N8" s="2">
         <v>0.10532407407407407</v>
       </c>
-      <c r="O8" s="1">
+      <c r="O8" s="27">
         <v>12.6</v>
       </c>
       <c r="P8" s="1">
@@ -19597,7 +19767,7 @@
       <c r="T8" s="2">
         <v>0.4417476851851852</v>
       </c>
-      <c r="U8" s="1">
+      <c r="U8" s="27">
         <v>15.925000000000001</v>
       </c>
       <c r="V8" s="1">
@@ -19612,7 +19782,7 @@
       <c r="Z8" s="2">
         <v>0.47152777777777777</v>
       </c>
-      <c r="AA8" s="1">
+      <c r="AA8" s="27">
         <v>16.100000000000001</v>
       </c>
       <c r="AB8" s="1">
@@ -19627,7 +19797,7 @@
       <c r="AF8" s="2">
         <v>8.4108796296296293E-2</v>
       </c>
-      <c r="AG8" s="1">
+      <c r="AG8" s="27">
         <v>10.092000000000001</v>
       </c>
       <c r="AH8" s="1">
@@ -19642,7 +19812,7 @@
       <c r="AL8" s="2">
         <v>0.46912037037037035</v>
       </c>
-      <c r="AM8" s="1">
+      <c r="AM8" s="27">
         <v>9.3919999999999995</v>
       </c>
       <c r="AN8" s="1">
@@ -19659,7 +19829,7 @@
       <c r="B9" s="2">
         <v>0.49877314814814816</v>
       </c>
-      <c r="C9" s="1">
+      <c r="C9" s="27">
         <v>12.134</v>
       </c>
       <c r="D9" s="1">
@@ -19674,7 +19844,7 @@
       <c r="H9" s="2">
         <v>7.962962962962962E-2</v>
       </c>
-      <c r="I9" s="1">
+      <c r="I9" s="27">
         <v>13.532999999999999</v>
       </c>
       <c r="J9" s="1">
@@ -19689,7 +19859,7 @@
       <c r="N9" s="2">
         <v>0.10543981481481481</v>
       </c>
-      <c r="O9" s="1">
+      <c r="O9" s="27">
         <v>11.667</v>
       </c>
       <c r="P9" s="1">
@@ -19704,7 +19874,7 @@
       <c r="T9" s="2">
         <v>0.44184027777777773</v>
       </c>
-      <c r="U9" s="1">
+      <c r="U9" s="27">
         <v>14</v>
       </c>
       <c r="V9" s="1">
@@ -19719,7 +19889,7 @@
       <c r="Z9" s="2">
         <v>0.47164351851851855</v>
       </c>
-      <c r="AA9" s="1">
+      <c r="AA9" s="27">
         <v>13.708</v>
       </c>
       <c r="AB9" s="1">
@@ -19734,7 +19904,7 @@
       <c r="AF9" s="2">
         <v>8.414351851851852E-2</v>
       </c>
-      <c r="AG9" s="1">
+      <c r="AG9" s="27">
         <v>10.442</v>
       </c>
       <c r="AH9" s="1">
@@ -19749,7 +19919,7 @@
       <c r="AL9" s="2">
         <v>0.46915509259259264</v>
       </c>
-      <c r="AM9" s="1">
+      <c r="AM9" s="27">
         <v>9.3919999999999995</v>
       </c>
       <c r="AN9" s="1">
@@ -19766,7 +19936,7 @@
       <c r="B10" s="2">
         <v>0.49890046296296298</v>
       </c>
-      <c r="C10" s="1">
+      <c r="C10" s="27">
         <v>11.959</v>
       </c>
       <c r="D10" s="1">
@@ -19781,7 +19951,7 @@
       <c r="H10" s="2">
         <v>7.9745370370370369E-2</v>
       </c>
-      <c r="I10" s="1">
+      <c r="I10" s="27">
         <v>13.708</v>
       </c>
       <c r="J10" s="1">
@@ -19796,7 +19966,7 @@
       <c r="N10" s="2">
         <v>0.10555555555555556</v>
       </c>
-      <c r="O10" s="1">
+      <c r="O10" s="27">
         <v>13.242000000000001</v>
       </c>
       <c r="P10" s="1">
@@ -19811,7 +19981,7 @@
       <c r="T10" s="2">
         <v>0.44195601851851851</v>
       </c>
-      <c r="U10" s="1">
+      <c r="U10" s="27">
         <v>11.782999999999999</v>
       </c>
       <c r="V10" s="1">
@@ -19826,7 +19996,7 @@
       <c r="Z10" s="2">
         <v>0.47175925925925927</v>
       </c>
-      <c r="AA10" s="1">
+      <c r="AA10" s="27">
         <v>12.483000000000001</v>
       </c>
       <c r="AB10" s="1">
@@ -19841,7 +20011,7 @@
       <c r="AF10" s="2">
         <v>8.4178240740740748E-2</v>
       </c>
-      <c r="AG10" s="1">
+      <c r="AG10" s="27">
         <v>10.617000000000001</v>
       </c>
       <c r="AH10" s="1">
@@ -19856,7 +20026,7 @@
       <c r="AL10" s="2">
         <v>0.46918981481481481</v>
       </c>
-      <c r="AM10" s="1">
+      <c r="AM10" s="27">
         <v>9.0419999999999998</v>
       </c>
       <c r="AN10" s="1">
@@ -19873,7 +20043,7 @@
       <c r="B11" s="2">
         <v>0.4990046296296296</v>
       </c>
-      <c r="C11" s="1">
+      <c r="C11" s="27">
         <v>11.959</v>
       </c>
       <c r="D11" s="1">
@@ -19888,7 +20058,7 @@
       <c r="H11" s="2">
         <v>7.9861111111111105E-2</v>
       </c>
-      <c r="I11" s="1">
+      <c r="I11" s="27">
         <v>12.775</v>
       </c>
       <c r="J11" s="1">
@@ -19903,7 +20073,7 @@
       <c r="N11" s="2">
         <v>0.10567129629629629</v>
       </c>
-      <c r="O11" s="1">
+      <c r="O11" s="27">
         <v>12.775</v>
       </c>
       <c r="P11" s="1">
@@ -19918,7 +20088,7 @@
       <c r="T11" s="2">
         <v>0.44208333333333333</v>
       </c>
-      <c r="U11" s="1">
+      <c r="U11" s="27">
         <v>10.558</v>
       </c>
       <c r="V11" s="1">
@@ -19933,7 +20103,7 @@
       <c r="Z11" s="2">
         <v>0.47187499999999999</v>
       </c>
-      <c r="AA11" s="1">
+      <c r="AA11" s="27">
         <v>11.375</v>
       </c>
       <c r="AB11" s="1">
@@ -19948,7 +20118,7 @@
       <c r="AF11" s="2">
         <v>8.4212962962962976E-2</v>
       </c>
-      <c r="AG11" s="1">
+      <c r="AG11" s="27">
         <v>10.442</v>
       </c>
       <c r="AH11" s="1">
@@ -19963,7 +20133,7 @@
       <c r="AL11" s="2">
         <v>0.46922453703703698</v>
       </c>
-      <c r="AM11" s="1">
+      <c r="AM11" s="27">
         <v>8.6920000000000002</v>
       </c>
       <c r="AN11" s="1">
@@ -19980,7 +20150,7 @@
       <c r="B12" s="2">
         <v>0.49912037037037038</v>
       </c>
-      <c r="C12" s="1">
+      <c r="C12" s="27">
         <v>11.784000000000001</v>
       </c>
       <c r="D12" s="1">
@@ -19995,7 +20165,7 @@
       <c r="H12" s="2">
         <v>7.9976851851851841E-2</v>
       </c>
-      <c r="I12" s="1">
+      <c r="I12" s="27">
         <v>12.132999999999999</v>
       </c>
       <c r="J12" s="1">
@@ -20010,7 +20180,7 @@
       <c r="N12" s="2">
         <v>0.10578703703703703</v>
       </c>
-      <c r="O12" s="1">
+      <c r="O12" s="27">
         <v>12.132999999999999</v>
       </c>
       <c r="P12" s="1">
@@ -20025,7 +20195,7 @@
       <c r="T12" s="2">
         <v>0.4422106481481482</v>
       </c>
-      <c r="U12" s="1">
+      <c r="U12" s="27">
         <v>10.382999999999999</v>
       </c>
       <c r="V12" s="1">
@@ -20040,7 +20210,7 @@
       <c r="Z12" s="2">
         <v>0.47199074074074071</v>
       </c>
-      <c r="AA12" s="1">
+      <c r="AA12" s="27">
         <v>10.558</v>
       </c>
       <c r="AB12" s="1">
@@ -20055,7 +20225,7 @@
       <c r="AF12" s="2">
         <v>8.4247685185185175E-2</v>
       </c>
-      <c r="AG12" s="1">
+      <c r="AG12" s="27">
         <v>10.092000000000001</v>
       </c>
       <c r="AH12" s="1">
@@ -20070,7 +20240,7 @@
       <c r="AL12" s="2">
         <v>0.46925925925925926</v>
       </c>
-      <c r="AM12" s="1">
+      <c r="AM12" s="27">
         <v>8.4580000000000002</v>
       </c>
       <c r="AN12" s="1">
@@ -20087,7 +20257,7 @@
       <c r="B13" s="2">
         <v>0.49923611111111116</v>
       </c>
-      <c r="C13" s="1">
+      <c r="C13" s="27">
         <v>11.959</v>
       </c>
       <c r="D13" s="1">
@@ -20102,7 +20272,7 @@
       <c r="H13" s="2">
         <v>8.009259259259259E-2</v>
       </c>
-      <c r="I13" s="1">
+      <c r="I13" s="27">
         <v>12.132999999999999</v>
       </c>
       <c r="J13" s="1">
@@ -20117,7 +20287,7 @@
       <c r="N13" s="2">
         <v>0.10590277777777778</v>
       </c>
-      <c r="O13" s="1">
+      <c r="O13" s="27">
         <v>11.958</v>
       </c>
       <c r="P13" s="1">
@@ -20132,7 +20302,7 @@
       <c r="T13" s="2">
         <v>0.44232638888888887</v>
       </c>
-      <c r="U13" s="1">
+      <c r="U13" s="27">
         <v>9.9160000000000004</v>
       </c>
       <c r="V13" s="1">
@@ -20147,7 +20317,7 @@
       <c r="Z13" s="2">
         <v>0.47210648148148149</v>
       </c>
-      <c r="AA13" s="1">
+      <c r="AA13" s="27">
         <v>10.85</v>
       </c>
       <c r="AB13" s="1">
@@ -20162,7 +20332,7 @@
       <c r="AF13" s="2">
         <v>8.4282407407407403E-2</v>
       </c>
-      <c r="AG13" s="1">
+      <c r="AG13" s="27">
         <v>9.9169999999999998</v>
       </c>
       <c r="AH13" s="1">
@@ -20177,7 +20347,7 @@
       <c r="AL13" s="2">
         <v>0.46929398148148144</v>
       </c>
-      <c r="AM13" s="1">
+      <c r="AM13" s="27">
         <v>8.2829999999999995</v>
       </c>
       <c r="AN13" s="1">
@@ -20194,7 +20364,7 @@
       <c r="B14" s="2">
         <v>0.49935185185185182</v>
       </c>
-      <c r="C14" s="1">
+      <c r="C14" s="27">
         <v>11.667</v>
       </c>
       <c r="D14" s="1">
@@ -20209,7 +20379,7 @@
       <c r="H14" s="2">
         <v>8.020833333333334E-2</v>
       </c>
-      <c r="I14" s="1">
+      <c r="I14" s="27">
         <v>11.958</v>
       </c>
       <c r="J14" s="1">
@@ -20224,7 +20394,7 @@
       <c r="N14" s="2">
         <v>0.10601851851851851</v>
       </c>
-      <c r="O14" s="1">
+      <c r="O14" s="27">
         <v>11.317</v>
       </c>
       <c r="P14" s="1">
@@ -20239,7 +20409,7 @@
       <c r="T14" s="2">
         <v>0.44244212962962964</v>
       </c>
-      <c r="U14" s="1">
+      <c r="U14" s="27">
         <v>9.7409999999999997</v>
       </c>
       <c r="V14" s="1">
@@ -20254,7 +20424,7 @@
       <c r="Z14" s="2">
         <v>0.47222222222222227</v>
       </c>
-      <c r="AA14" s="1">
+      <c r="AA14" s="27">
         <v>10.85</v>
       </c>
       <c r="AB14" s="1">
@@ -20271,7 +20441,7 @@
       <c r="B15" s="2">
         <v>0.49945601851851856</v>
       </c>
-      <c r="C15" s="1">
+      <c r="C15" s="27">
         <v>11.492000000000001</v>
       </c>
       <c r="D15" s="1">
@@ -20286,7 +20456,7 @@
       <c r="H15" s="2">
         <v>8.0324074074074062E-2</v>
       </c>
-      <c r="I15" s="1">
+      <c r="I15" s="27">
         <v>11.317</v>
       </c>
       <c r="J15" s="1">
@@ -20301,7 +20471,7 @@
       <c r="N15" s="2">
         <v>0.10613425925925928</v>
       </c>
-      <c r="O15" s="1">
+      <c r="O15" s="27">
         <v>11.782999999999999</v>
       </c>
       <c r="P15" s="1">
@@ -20316,7 +20486,7 @@
       <c r="Z15" s="2">
         <v>0.47233796296296293</v>
       </c>
-      <c r="AA15" s="1">
+      <c r="AA15" s="27">
         <v>10.382999999999999</v>
       </c>
       <c r="AB15" s="1">
@@ -20333,7 +20503,7 @@
       <c r="B16" s="2">
         <v>0.49958333333333332</v>
       </c>
-      <c r="C16" s="1">
+      <c r="C16" s="27">
         <v>11.667</v>
       </c>
       <c r="D16" s="1">
@@ -20348,7 +20518,7 @@
       <c r="H16" s="2">
         <v>8.0439814814814811E-2</v>
       </c>
-      <c r="I16" s="1">
+      <c r="I16" s="27">
         <v>11.667</v>
       </c>
       <c r="J16" s="1">
@@ -20365,7 +20535,7 @@
       <c r="H17" s="2">
         <v>8.0555555555555561E-2</v>
       </c>
-      <c r="I17" s="1">
+      <c r="I17" s="27">
         <v>11.667</v>
       </c>
       <c r="J17" s="1">
@@ -20382,7 +20552,7 @@
       <c r="H18" s="2">
         <v>8.0671296296296297E-2</v>
       </c>
-      <c r="I18" s="1">
+      <c r="I18" s="27">
         <v>11.492000000000001</v>
       </c>
       <c r="J18" s="1">
@@ -20405,4 +20575,1745 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F3F9C6C4-043C-4DB8-AE02-89656D936DC4}">
+  <dimension ref="A1:G90"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="23.85546875" customWidth="1"/>
+    <col min="2" max="2" width="11.7109375" customWidth="1"/>
+    <col min="3" max="3" width="12.28515625" customWidth="1"/>
+    <col min="4" max="4" width="12.140625" customWidth="1"/>
+    <col min="5" max="5" width="11.28515625" customWidth="1"/>
+    <col min="6" max="6" width="12.42578125" customWidth="1"/>
+    <col min="7" max="7" width="11.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" s="16" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="C1" s="17" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1" s="17" t="s">
+        <v>23</v>
+      </c>
+      <c r="E1" s="18" t="s">
+        <v>19</v>
+      </c>
+      <c r="F1" s="17" t="s">
+        <v>24</v>
+      </c>
+      <c r="G1" s="17" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" s="20">
+        <v>167.04416761041898</v>
+      </c>
+      <c r="C2" s="20">
+        <v>10.974524206225087</v>
+      </c>
+      <c r="D2" s="23">
+        <v>2.64</v>
+      </c>
+      <c r="E2" s="8">
+        <v>1.003934430437827E-2</v>
+      </c>
+      <c r="F2" s="8">
+        <v>2.45715E-2</v>
+      </c>
+      <c r="G2" s="9">
+        <v>0.49802083333333336</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" s="20">
+        <v>145.07862045000454</v>
+      </c>
+      <c r="C3" s="20">
+        <v>12.330497071523524</v>
+      </c>
+      <c r="D3" s="23">
+        <v>2.3839999999999999</v>
+      </c>
+      <c r="E3" s="8">
+        <v>2.2338385851655443E-2</v>
+      </c>
+      <c r="F3" s="8">
+        <v>1.7498300000000022E-2</v>
+      </c>
+      <c r="G3" s="9">
+        <v>0.49815972222222221</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" s="20">
+        <v>76.137884872824614</v>
+      </c>
+      <c r="C4" s="20"/>
+      <c r="D4" s="23">
+        <v>2.2839999999999998</v>
+      </c>
+      <c r="E4" s="8">
+        <v>9.8099758295017991E-3</v>
+      </c>
+      <c r="F4" s="8">
+        <v>2.1034899999999995E-2</v>
+      </c>
+      <c r="G4" s="9">
+        <v>0.49828703703703708</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="20">
+        <v>47.967684928048556</v>
+      </c>
+      <c r="C5" s="20">
+        <v>4.9671491115903788</v>
+      </c>
+      <c r="D5" s="23">
+        <v>2.423</v>
+      </c>
+      <c r="E5" s="8">
+        <v>1.031870116219955E-2</v>
+      </c>
+      <c r="F5" s="8">
+        <v>2.9876399999999997E-2</v>
+      </c>
+      <c r="G5" s="9">
+        <v>0.49840277777777775</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" s="20">
+        <v>67.326074308037519</v>
+      </c>
+      <c r="C6" s="20">
+        <v>8.8903535000293825</v>
+      </c>
+      <c r="D6" s="23">
+        <v>2.488</v>
+      </c>
+      <c r="E6" s="8">
+        <v>6.2101564483107649E-3</v>
+      </c>
+      <c r="F6" s="8">
+        <v>2.6339799999999997E-2</v>
+      </c>
+      <c r="G6" s="9">
+        <v>0.49853009259259262</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" s="20">
+        <v>61.268421924159554</v>
+      </c>
+      <c r="C7" s="20"/>
+      <c r="D7" s="23">
+        <v>2.4729999999999999</v>
+      </c>
+      <c r="E7" s="8">
+        <v>5.2426659536415413E-3</v>
+      </c>
+      <c r="F7" s="8">
+        <v>2.8108099999999997E-2</v>
+      </c>
+      <c r="G7" s="9">
+        <v>0.49865740740740744</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" s="20">
+        <v>40.782355389096857</v>
+      </c>
+      <c r="C8" s="20"/>
+      <c r="D8" s="23">
+        <v>2.3140000000000001</v>
+      </c>
+      <c r="E8" s="8">
+        <v>3.2996877945532998E-3</v>
+      </c>
+      <c r="F8" s="8">
+        <v>2.8108099999999997E-2</v>
+      </c>
+      <c r="G8" s="9">
+        <v>0.49877314814814816</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9" s="20">
+        <v>43.350237199411083</v>
+      </c>
+      <c r="C9" s="20"/>
+      <c r="D9" s="23">
+        <v>2.4020000000000001</v>
+      </c>
+      <c r="E9" s="8">
+        <v>2.600539216633088E-3</v>
+      </c>
+      <c r="F9" s="8">
+        <v>2.9876399999999997E-2</v>
+      </c>
+      <c r="G9" s="9">
+        <v>0.49890046296296298</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B10" s="20">
+        <v>37.341299477221838</v>
+      </c>
+      <c r="C10" s="20"/>
+      <c r="D10" s="23">
+        <v>2.278</v>
+      </c>
+      <c r="E10" s="8">
+        <v>2.618500653426792E-3</v>
+      </c>
+      <c r="F10" s="8">
+        <v>2.4571499999999996E-2</v>
+      </c>
+      <c r="G10" s="9">
+        <v>0.4990046296296296</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B11" s="20">
+        <v>22.213081036610511</v>
+      </c>
+      <c r="C11" s="20"/>
+      <c r="D11" s="23">
+        <v>2.2730000000000001</v>
+      </c>
+      <c r="E11" s="8">
+        <v>4.3689279273505278E-3</v>
+      </c>
+      <c r="F11" s="8">
+        <v>2.8108099999999997E-2</v>
+      </c>
+      <c r="G11" s="9">
+        <v>0.49912037037037038</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B12" s="20">
+        <v>20.673116679070553</v>
+      </c>
+      <c r="C12" s="20"/>
+      <c r="D12" s="23">
+        <v>2.3010000000000002</v>
+      </c>
+      <c r="E12" s="8">
+        <v>3.1173927792587626E-3</v>
+      </c>
+      <c r="F12" s="8">
+        <v>2.6339799999999997E-2</v>
+      </c>
+      <c r="G12" s="9">
+        <v>0.49923611111111116</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" s="20">
+        <v>12.548101054040499</v>
+      </c>
+      <c r="C13" s="20">
+        <v>3.2415982125782183</v>
+      </c>
+      <c r="D13" s="23">
+        <v>2.3130000000000002</v>
+      </c>
+      <c r="E13" s="8">
+        <v>2.5711583887521052E-3</v>
+      </c>
+      <c r="F13" s="8">
+        <v>1.9266599999999995E-2</v>
+      </c>
+      <c r="G13" s="9">
+        <v>0.49935185185185182</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B14" s="20">
+        <v>10.726957669774698</v>
+      </c>
+      <c r="C14" s="20"/>
+      <c r="D14" s="23">
+        <v>2.3079999999999998</v>
+      </c>
+      <c r="E14" s="8">
+        <v>2.600539216633088E-3</v>
+      </c>
+      <c r="F14" s="8">
+        <v>2.1034899999999995E-2</v>
+      </c>
+      <c r="G14" s="9">
+        <v>0.49945601851851856</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B15" s="20">
+        <v>6.584362139917884</v>
+      </c>
+      <c r="C15" s="20"/>
+      <c r="D15" s="23">
+        <v>2.214</v>
+      </c>
+      <c r="E15" s="8">
+        <v>2.2886277341208801E-3</v>
+      </c>
+      <c r="F15" s="8">
+        <v>2.2803199999999996E-2</v>
+      </c>
+      <c r="G15" s="9">
+        <v>0.49958333333333332</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="B16" s="21">
+        <v>22.819885900570469</v>
+      </c>
+      <c r="C16" s="21">
+        <v>3.3278897667339491</v>
+      </c>
+      <c r="D16" s="24">
+        <v>2.718</v>
+      </c>
+      <c r="E16" s="11"/>
+      <c r="F16" s="11"/>
+      <c r="G16" s="12">
+        <v>0.57892361111111112</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="B17" s="21">
+        <v>66.633761105626817</v>
+      </c>
+      <c r="C17" s="21">
+        <v>6.6628506349267198</v>
+      </c>
+      <c r="D17" s="24">
+        <v>2.6819999999999999</v>
+      </c>
+      <c r="E17" s="11"/>
+      <c r="F17" s="11"/>
+      <c r="G17" s="12">
+        <v>0.57905092592592589</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="B18" s="21">
+        <v>162.54186065506821</v>
+      </c>
+      <c r="C18" s="21">
+        <v>12.041210880553001</v>
+      </c>
+      <c r="D18" s="24">
+        <v>2.6440000000000001</v>
+      </c>
+      <c r="E18" s="11"/>
+      <c r="F18" s="11"/>
+      <c r="G18" s="12">
+        <v>0.57916666666666672</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="B19" s="21">
+        <v>89.561960592737421</v>
+      </c>
+      <c r="C19" s="21"/>
+      <c r="D19" s="24">
+        <v>2.7519999999999998</v>
+      </c>
+      <c r="E19" s="11"/>
+      <c r="F19" s="11"/>
+      <c r="G19" s="12">
+        <v>0.57928240740740744</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="B20" s="21">
+        <v>87.538194731191894</v>
+      </c>
+      <c r="C20" s="21">
+        <v>8.058197301683574</v>
+      </c>
+      <c r="D20" s="24">
+        <v>2.8079999999999998</v>
+      </c>
+      <c r="E20" s="11"/>
+      <c r="F20" s="11"/>
+      <c r="G20" s="12">
+        <v>0.57939814814814816</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="B21" s="21">
+        <v>67.359667359667327</v>
+      </c>
+      <c r="C21" s="21"/>
+      <c r="D21" s="24">
+        <v>3.0089999999999999</v>
+      </c>
+      <c r="E21" s="11"/>
+      <c r="F21" s="11"/>
+      <c r="G21" s="12">
+        <v>0.57951388888888888</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A22" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="B22" s="21">
+        <v>61.637080867850159</v>
+      </c>
+      <c r="C22" s="21"/>
+      <c r="D22" s="24">
+        <v>2.7839999999999998</v>
+      </c>
+      <c r="E22" s="11"/>
+      <c r="F22" s="11"/>
+      <c r="G22" s="12">
+        <v>0.57962962962962961</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A23" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="B23" s="21">
+        <v>37.633968747443511</v>
+      </c>
+      <c r="C23" s="21">
+        <v>5.0565465878568743</v>
+      </c>
+      <c r="D23" s="24">
+        <v>2.7559999999999998</v>
+      </c>
+      <c r="E23" s="11"/>
+      <c r="F23" s="11"/>
+      <c r="G23" s="12">
+        <v>0.57974537037037033</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A24" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="B24" s="21">
+        <v>49.685326266975864</v>
+      </c>
+      <c r="C24" s="21">
+        <v>3.7364280370951577</v>
+      </c>
+      <c r="D24" s="24">
+        <v>2.8039999999999998</v>
+      </c>
+      <c r="E24" s="11"/>
+      <c r="F24" s="11"/>
+      <c r="G24" s="12">
+        <v>0.57986111111111116</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A25" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="B25" s="21">
+        <v>30.50037095045758</v>
+      </c>
+      <c r="C25" s="21"/>
+      <c r="D25" s="24">
+        <v>2.8039999999999998</v>
+      </c>
+      <c r="E25" s="11"/>
+      <c r="F25" s="11"/>
+      <c r="G25" s="12">
+        <v>0.57997685185185188</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A26" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="B26" s="21">
+        <v>27.990450316950803</v>
+      </c>
+      <c r="C26" s="21"/>
+      <c r="D26" s="24">
+        <v>2.8639999999999999</v>
+      </c>
+      <c r="E26" s="11"/>
+      <c r="F26" s="11"/>
+      <c r="G26" s="12">
+        <v>0.5800925925925926</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A27" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="B27" s="21">
+        <v>16.572754391779927</v>
+      </c>
+      <c r="C27" s="21">
+        <v>2.7714442809806075</v>
+      </c>
+      <c r="D27" s="24">
+        <v>2.76</v>
+      </c>
+      <c r="E27" s="11"/>
+      <c r="F27" s="11"/>
+      <c r="G27" s="12">
+        <v>0.58020833333333333</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A28" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="B28" s="21">
+        <v>18.36853970109383</v>
+      </c>
+      <c r="C28" s="21"/>
+      <c r="D28" s="24">
+        <v>2.7690000000000001</v>
+      </c>
+      <c r="E28" s="11"/>
+      <c r="F28" s="11"/>
+      <c r="G28" s="12">
+        <v>0.58032407407407405</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A29" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="B29" s="21">
+        <v>6.4583837894566489</v>
+      </c>
+      <c r="C29" s="21"/>
+      <c r="D29" s="24">
+        <v>2.7410000000000001</v>
+      </c>
+      <c r="E29" s="11"/>
+      <c r="F29" s="11"/>
+      <c r="G29" s="12">
+        <v>0.58043981481481477</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A30" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="B30" s="21">
+        <v>11.361791916896708</v>
+      </c>
+      <c r="C30" s="21"/>
+      <c r="D30" s="24">
+        <v>2.7519999999999998</v>
+      </c>
+      <c r="E30" s="11"/>
+      <c r="F30" s="11"/>
+      <c r="G30" s="12">
+        <v>0.5805555555555556</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A31" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="B31" s="21">
+        <v>11.501807426881468</v>
+      </c>
+      <c r="C31" s="21"/>
+      <c r="D31" s="24">
+        <v>2.7389999999999999</v>
+      </c>
+      <c r="E31" s="11"/>
+      <c r="F31" s="11"/>
+      <c r="G31" s="12">
+        <v>0.58067129629629632</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A32" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="B32" s="22">
+        <v>52.169592580324611</v>
+      </c>
+      <c r="C32" s="22">
+        <v>4.595228517796305</v>
+      </c>
+      <c r="D32" s="25">
+        <v>2.8980000000000001</v>
+      </c>
+      <c r="E32" s="14"/>
+      <c r="F32" s="14"/>
+      <c r="G32" s="15">
+        <v>0.60474537037037035</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A33" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="B33" s="22">
+        <v>174.67613873798578</v>
+      </c>
+      <c r="C33" s="22">
+        <v>10.930144320508324</v>
+      </c>
+      <c r="D33" s="25">
+        <v>2.7160000000000002</v>
+      </c>
+      <c r="E33" s="14"/>
+      <c r="F33" s="14"/>
+      <c r="G33" s="15">
+        <v>0.60486111111111107</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A34" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="B34" s="22">
+        <v>78.177538668460016</v>
+      </c>
+      <c r="C34" s="22"/>
+      <c r="D34" s="25">
+        <v>2.7010000000000001</v>
+      </c>
+      <c r="E34" s="14"/>
+      <c r="F34" s="14"/>
+      <c r="G34" s="15">
+        <v>0.6049768518518519</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A35" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="B35" s="22">
+        <v>74.758733179285102</v>
+      </c>
+      <c r="C35" s="22">
+        <v>8.9789966308393812</v>
+      </c>
+      <c r="D35" s="25">
+        <v>2.7810000000000001</v>
+      </c>
+      <c r="E35" s="14"/>
+      <c r="F35" s="14"/>
+      <c r="G35" s="15">
+        <v>0.60509259259259263</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A36" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="B36" s="22">
+        <v>52.974735126324418</v>
+      </c>
+      <c r="C36" s="22"/>
+      <c r="D36" s="25">
+        <v>2.831</v>
+      </c>
+      <c r="E36" s="14"/>
+      <c r="F36" s="14"/>
+      <c r="G36" s="15">
+        <v>0.60520833333333335</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A37" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="B37" s="22">
+        <v>40.183696900114938</v>
+      </c>
+      <c r="C37" s="22"/>
+      <c r="D37" s="25">
+        <v>2.7629999999999999</v>
+      </c>
+      <c r="E37" s="14"/>
+      <c r="F37" s="14"/>
+      <c r="G37" s="15">
+        <v>0.60532407407407407</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A38" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="B38" s="22">
+        <v>43.398430979802896</v>
+      </c>
+      <c r="C38" s="22">
+        <v>4.599424686865893</v>
+      </c>
+      <c r="D38" s="25">
+        <v>2.8140000000000001</v>
+      </c>
+      <c r="E38" s="14"/>
+      <c r="F38" s="14"/>
+      <c r="G38" s="15">
+        <v>0.60543981481481479</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A39" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="B39" s="22">
+        <v>77.334430275606678</v>
+      </c>
+      <c r="C39" s="22"/>
+      <c r="D39" s="25">
+        <v>2.7469999999999999</v>
+      </c>
+      <c r="E39" s="14"/>
+      <c r="F39" s="14"/>
+      <c r="G39" s="15">
+        <v>0.60555555555555551</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A40" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="B40" s="22">
+        <v>58.595361888256129</v>
+      </c>
+      <c r="C40" s="22"/>
+      <c r="D40" s="25">
+        <v>2.7410000000000001</v>
+      </c>
+      <c r="E40" s="14"/>
+      <c r="F40" s="14"/>
+      <c r="G40" s="15">
+        <v>0.60567129629629635</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A41" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="B41" s="22">
+        <v>23.829087921117384</v>
+      </c>
+      <c r="C41" s="22"/>
+      <c r="D41" s="25">
+        <v>2.7749999999999999</v>
+      </c>
+      <c r="E41" s="14"/>
+      <c r="F41" s="14"/>
+      <c r="G41" s="15">
+        <v>0.60578703703703707</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A42" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="B42" s="22">
+        <v>26.223059903302538</v>
+      </c>
+      <c r="C42" s="22"/>
+      <c r="D42" s="25">
+        <v>2.7330000000000001</v>
+      </c>
+      <c r="E42" s="14"/>
+      <c r="F42" s="14"/>
+      <c r="G42" s="15">
+        <v>0.60590277777777779</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A43" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="B43" s="22">
+        <v>17.731993582707005</v>
+      </c>
+      <c r="C43" s="22">
+        <v>3.2584248138189293</v>
+      </c>
+      <c r="D43" s="25">
+        <v>2.7559999999999998</v>
+      </c>
+      <c r="E43" s="14"/>
+      <c r="F43" s="14"/>
+      <c r="G43" s="15">
+        <v>0.60601851851851851</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A44" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="B44" s="22">
+        <v>18.922254216371837</v>
+      </c>
+      <c r="C44" s="22"/>
+      <c r="D44" s="25">
+        <v>2.7850000000000001</v>
+      </c>
+      <c r="E44" s="14"/>
+      <c r="F44" s="14"/>
+      <c r="G44" s="15">
+        <v>0.60613425925925923</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A45" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B45" s="19">
+        <v>70.55388857351403</v>
+      </c>
+      <c r="C45" s="19">
+        <v>8.3572964290100931</v>
+      </c>
+      <c r="D45" s="26">
+        <v>2.1829999999999998</v>
+      </c>
+      <c r="E45" s="6"/>
+      <c r="F45" s="6"/>
+      <c r="G45" s="5">
+        <v>0.4397685185185185</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A46" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B46" s="19">
+        <v>287.82894736842087</v>
+      </c>
+      <c r="C46" s="19">
+        <v>24.660150936233205</v>
+      </c>
+      <c r="D46" s="26">
+        <v>2.1179999999999999</v>
+      </c>
+      <c r="E46" s="6"/>
+      <c r="F46" s="6"/>
+      <c r="G46" s="5">
+        <v>0.44150462962962966</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A47" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B47" s="19">
+        <v>200.049804930688</v>
+      </c>
+      <c r="C47" s="19">
+        <v>16.604665163366334</v>
+      </c>
+      <c r="D47" s="26">
+        <v>2.073</v>
+      </c>
+      <c r="E47" s="6"/>
+      <c r="F47" s="6"/>
+      <c r="G47" s="5">
+        <v>0.44156250000000002</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A48" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B48" s="19">
+        <v>112.46027218645594</v>
+      </c>
+      <c r="C48" s="19">
+        <v>10.359493646922049</v>
+      </c>
+      <c r="D48" s="26">
+        <v>2.0289999999999999</v>
+      </c>
+      <c r="E48" s="6"/>
+      <c r="F48" s="6"/>
+      <c r="G48" s="5">
+        <v>0.44162037037037033</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A49" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B49" s="19">
+        <v>111.46627325629046</v>
+      </c>
+      <c r="C49" s="19"/>
+      <c r="D49" s="26">
+        <v>2.0779999999999998</v>
+      </c>
+      <c r="E49" s="6"/>
+      <c r="F49" s="6"/>
+      <c r="G49" s="5">
+        <v>0.44167824074074075</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A50" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B50" s="19">
+        <v>79.809116340299596</v>
+      </c>
+      <c r="C50" s="19">
+        <v>9.283897155762066</v>
+      </c>
+      <c r="D50" s="26">
+        <v>2.1640000000000001</v>
+      </c>
+      <c r="E50" s="6"/>
+      <c r="F50" s="6"/>
+      <c r="G50" s="5">
+        <v>0.4417476851851852</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A51" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B51" s="19">
+        <v>80.492813141683797</v>
+      </c>
+      <c r="C51" s="19"/>
+      <c r="D51" s="26">
+        <v>2.1720000000000002</v>
+      </c>
+      <c r="E51" s="6"/>
+      <c r="F51" s="6"/>
+      <c r="G51" s="5">
+        <v>0.44184027777777773</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A52" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B52" s="19">
+        <v>69.473161855926037</v>
+      </c>
+      <c r="C52" s="19"/>
+      <c r="D52" s="26">
+        <v>2.3029999999999999</v>
+      </c>
+      <c r="E52" s="6"/>
+      <c r="F52" s="6"/>
+      <c r="G52" s="5">
+        <v>0.44195601851851851</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A53" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B53" s="19">
+        <v>54.027504911591542</v>
+      </c>
+      <c r="C53" s="19"/>
+      <c r="D53" s="26">
+        <v>2.2890000000000001</v>
+      </c>
+      <c r="E53" s="6"/>
+      <c r="F53" s="6"/>
+      <c r="G53" s="5">
+        <v>0.44208333333333333</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A54" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B54" s="19">
+        <v>44.106836559666647</v>
+      </c>
+      <c r="C54" s="19">
+        <v>5.2546784274057234</v>
+      </c>
+      <c r="D54" s="26">
+        <v>2.1890000000000001</v>
+      </c>
+      <c r="E54" s="6"/>
+      <c r="F54" s="6"/>
+      <c r="G54" s="5">
+        <v>0.4422106481481482</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A55" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B55" s="19">
+        <v>33.532346446389077</v>
+      </c>
+      <c r="C55" s="19"/>
+      <c r="D55" s="26">
+        <v>2.2829999999999999</v>
+      </c>
+      <c r="E55" s="6"/>
+      <c r="F55" s="6"/>
+      <c r="G55" s="5">
+        <v>0.44232638888888887</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A56" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B56" s="19">
+        <v>23.144321375433929</v>
+      </c>
+      <c r="C56" s="19"/>
+      <c r="D56" s="26">
+        <v>2.202</v>
+      </c>
+      <c r="E56" s="6"/>
+      <c r="F56" s="6"/>
+      <c r="G56" s="5">
+        <v>0.44244212962962964</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A57" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="B57" s="20">
+        <v>62.139769452449464</v>
+      </c>
+      <c r="C57" s="20">
+        <v>5.3161272316566057</v>
+      </c>
+      <c r="D57" s="23">
+        <v>2.6309999999999998</v>
+      </c>
+      <c r="E57" s="8">
+        <v>8.0744786331715737E-3</v>
+      </c>
+      <c r="F57" s="8">
+        <v>2.2803199999999996E-2</v>
+      </c>
+      <c r="G57" s="9">
+        <v>0.46828703703703706</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A58" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="B58" s="20">
+        <v>243.34662651582957</v>
+      </c>
+      <c r="C58" s="20">
+        <v>20.726107961901139</v>
+      </c>
+      <c r="D58" s="23">
+        <v>2.581</v>
+      </c>
+      <c r="E58" s="8">
+        <v>2.3321471582393793E-2</v>
+      </c>
+      <c r="F58" s="8">
+        <v>1.9266599999999995E-2</v>
+      </c>
+      <c r="G58" s="9">
+        <v>0.47123842592592591</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A59" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="B59" s="20">
+        <v>134.52914798206268</v>
+      </c>
+      <c r="C59" s="20"/>
+      <c r="D59" s="23">
+        <v>2.5630000000000002</v>
+      </c>
+      <c r="E59" s="8">
+        <v>1.9203510472240316E-2</v>
+      </c>
+      <c r="F59" s="8">
+        <v>2.2803199999999996E-2</v>
+      </c>
+      <c r="G59" s="9">
+        <v>0.47129629629629632</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A60" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="B60" s="20">
+        <v>135.40290620871883</v>
+      </c>
+      <c r="C60" s="20">
+        <v>11.667976217862849</v>
+      </c>
+      <c r="D60" s="23">
+        <v>2.6619999999999999</v>
+      </c>
+      <c r="E60" s="8">
+        <v>1.15146880608244E-2</v>
+      </c>
+      <c r="F60" s="8">
+        <v>2.2803199999999996E-2</v>
+      </c>
+      <c r="G60" s="9">
+        <v>0.47135416666666669</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A61" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="B61" s="20">
+        <v>99.901735997379532</v>
+      </c>
+      <c r="C61" s="20"/>
+      <c r="D61" s="23">
+        <v>2.6960000000000002</v>
+      </c>
+      <c r="E61" s="8">
+        <v>9.856082656835876E-3</v>
+      </c>
+      <c r="F61" s="8">
+        <v>2.1034899999999995E-2</v>
+      </c>
+      <c r="G61" s="9">
+        <v>0.47141203703703699</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A62" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="B62" s="20">
+        <v>98.606470540298261</v>
+      </c>
+      <c r="C62" s="20">
+        <v>6.6757924819308254</v>
+      </c>
+      <c r="D62" s="23">
+        <v>2.6989999999999998</v>
+      </c>
+      <c r="E62" s="8">
+        <v>1.16917712529308E-2</v>
+      </c>
+      <c r="F62" s="8">
+        <v>2.1034899999999995E-2</v>
+      </c>
+      <c r="G62" s="9">
+        <v>0.47152777777777777</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A63" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="B63" s="20">
+        <v>93.938898872733063</v>
+      </c>
+      <c r="C63" s="20"/>
+      <c r="D63" s="23">
+        <v>2.742</v>
+      </c>
+      <c r="E63" s="8">
+        <v>1.2283480760895546E-2</v>
+      </c>
+      <c r="F63" s="8">
+        <v>1.7498300000000022E-2</v>
+      </c>
+      <c r="G63" s="9">
+        <v>0.47164351851851855</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A64" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="B64" s="20">
+        <v>56.216392374124084</v>
+      </c>
+      <c r="C64" s="20"/>
+      <c r="D64" s="23">
+        <v>2.7610000000000001</v>
+      </c>
+      <c r="E64" s="8">
+        <v>8.7555621153478178E-3</v>
+      </c>
+      <c r="F64" s="8">
+        <v>2.4571499999999996E-2</v>
+      </c>
+      <c r="G64" s="9">
+        <v>0.47175925925925927</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A65" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="B65" s="20">
+        <v>56.813503499382371</v>
+      </c>
+      <c r="C65" s="20"/>
+      <c r="D65" s="23">
+        <v>2.8210000000000002</v>
+      </c>
+      <c r="E65" s="8">
+        <v>5.741883910742567E-3</v>
+      </c>
+      <c r="F65" s="8">
+        <v>2.4571499999999996E-2</v>
+      </c>
+      <c r="G65" s="9">
+        <v>0.47187499999999999</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A66" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="B66" s="20">
+        <v>48.527718374732594</v>
+      </c>
+      <c r="C66" s="20">
+        <v>5.6309098454195041</v>
+      </c>
+      <c r="D66" s="23">
+        <v>2.7829999999999999</v>
+      </c>
+      <c r="E66" s="8">
+        <v>4.5804950914437453E-3</v>
+      </c>
+      <c r="F66" s="8">
+        <v>2.6339799999999997E-2</v>
+      </c>
+      <c r="G66" s="9">
+        <v>0.47199074074074071</v>
+      </c>
+    </row>
+    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A67" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="B67" s="20">
+        <v>41.608876560333044</v>
+      </c>
+      <c r="C67" s="20"/>
+      <c r="D67" s="23">
+        <v>2.7559999999999998</v>
+      </c>
+      <c r="E67" s="8">
+        <v>4.0576794789688791E-3</v>
+      </c>
+      <c r="F67" s="8">
+        <v>2.1034899999999995E-2</v>
+      </c>
+      <c r="G67" s="9">
+        <v>0.47210648148148149</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A68" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="B68" s="20">
+        <v>27.029240724056002</v>
+      </c>
+      <c r="C68" s="20"/>
+      <c r="D68" s="23">
+        <v>2.883</v>
+      </c>
+      <c r="E68" s="8">
+        <v>3.3758505307597045E-3</v>
+      </c>
+      <c r="F68" s="8">
+        <v>2.2803199999999996E-2</v>
+      </c>
+      <c r="G68" s="9">
+        <v>0.47222222222222227</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A69" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="B69" s="20">
+        <v>22.118456623249024</v>
+      </c>
+      <c r="C69" s="20"/>
+      <c r="D69" s="23">
+        <v>2.84</v>
+      </c>
+      <c r="E69" s="8">
+        <v>3.4794954752049401E-3</v>
+      </c>
+      <c r="F69" s="8">
+        <v>2.4571499999999996E-2</v>
+      </c>
+      <c r="G69" s="9">
+        <v>0.47233796296296293</v>
+      </c>
+    </row>
+    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A70" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="B70" s="21">
+        <v>25.420254202541958</v>
+      </c>
+      <c r="C70" s="21">
+        <v>3.6469399778041134</v>
+      </c>
+      <c r="D70" s="24">
+        <v>2.9359999999999999</v>
+      </c>
+      <c r="E70" s="11"/>
+      <c r="F70" s="11"/>
+      <c r="G70" s="12">
+        <v>0.58261574074074074</v>
+      </c>
+    </row>
+    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A71" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="B71" s="21">
+        <v>9.0053213262383771</v>
+      </c>
+      <c r="C71" s="21"/>
+      <c r="D71" s="24">
+        <v>3.0289999999999999</v>
+      </c>
+      <c r="E71" s="11"/>
+      <c r="F71" s="11"/>
+      <c r="G71" s="12">
+        <v>0.5839699074074074</v>
+      </c>
+    </row>
+    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A72" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="B72" s="21">
+        <v>7.4868979286247752</v>
+      </c>
+      <c r="C72" s="21">
+        <v>2.3834166495325055</v>
+      </c>
+      <c r="D72" s="24">
+        <v>2.923</v>
+      </c>
+      <c r="E72" s="11"/>
+      <c r="F72" s="11"/>
+      <c r="G72" s="12">
+        <v>0.58400462962962962</v>
+      </c>
+    </row>
+    <row r="73" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A73" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="B73" s="21">
+        <v>4.9549921545958968</v>
+      </c>
+      <c r="C73" s="21"/>
+      <c r="D73" s="24">
+        <v>2.976</v>
+      </c>
+      <c r="E73" s="11"/>
+      <c r="F73" s="11"/>
+      <c r="G73" s="12">
+        <v>0.58403935185185185</v>
+      </c>
+    </row>
+    <row r="74" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A74" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="B74" s="21">
+        <v>7.3004542504865686</v>
+      </c>
+      <c r="C74" s="21">
+        <v>2.1756635953794543</v>
+      </c>
+      <c r="D74" s="24">
+        <v>3.641</v>
+      </c>
+      <c r="E74" s="11"/>
+      <c r="F74" s="11"/>
+      <c r="G74" s="12">
+        <v>0.58407407407407408</v>
+      </c>
+    </row>
+    <row r="75" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A75" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="B75" s="21">
+        <v>31.924724859279156</v>
+      </c>
+      <c r="C75" s="21"/>
+      <c r="D75" s="24">
+        <v>3.0539999999999998</v>
+      </c>
+      <c r="E75" s="11"/>
+      <c r="F75" s="11"/>
+      <c r="G75" s="12">
+        <v>0.58410879629629631</v>
+      </c>
+    </row>
+    <row r="76" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A76" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="B76" s="21">
+        <v>41.421588932151479</v>
+      </c>
+      <c r="C76" s="21"/>
+      <c r="D76" s="24">
+        <v>3.0379999999999998</v>
+      </c>
+      <c r="E76" s="11"/>
+      <c r="F76" s="11"/>
+      <c r="G76" s="12">
+        <v>0.58414351851851853</v>
+      </c>
+    </row>
+    <row r="77" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A77" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="B77" s="21">
+        <v>44.890630101208011</v>
+      </c>
+      <c r="C77" s="21">
+        <v>4.7777531047551749</v>
+      </c>
+      <c r="D77" s="24">
+        <v>3.5790000000000002</v>
+      </c>
+      <c r="E77" s="11"/>
+      <c r="F77" s="11"/>
+      <c r="G77" s="12">
+        <v>0.58417824074074076</v>
+      </c>
+    </row>
+    <row r="78" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A78" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="B78" s="21">
+        <v>33.18400530944087</v>
+      </c>
+      <c r="C78" s="21"/>
+      <c r="D78" s="24">
+        <v>3.1509999999999998</v>
+      </c>
+      <c r="E78" s="11"/>
+      <c r="F78" s="11"/>
+      <c r="G78" s="12">
+        <v>0.58421296296296299</v>
+      </c>
+    </row>
+    <row r="79" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A79" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="B79" s="21">
+        <v>25.368248772504021</v>
+      </c>
+      <c r="C79" s="21">
+        <v>4.932223506380244</v>
+      </c>
+      <c r="D79" s="24">
+        <v>3.0059999999999998</v>
+      </c>
+      <c r="E79" s="11"/>
+      <c r="F79" s="11"/>
+      <c r="G79" s="12">
+        <v>0.58424768518518522</v>
+      </c>
+    </row>
+    <row r="80" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A80" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="B80" s="21">
+        <v>6.545573555882795</v>
+      </c>
+      <c r="C80" s="21"/>
+      <c r="D80" s="24">
+        <v>3.5510000000000002</v>
+      </c>
+      <c r="E80" s="11"/>
+      <c r="F80" s="11"/>
+      <c r="G80" s="12">
+        <v>0.58428240740740744</v>
+      </c>
+    </row>
+    <row r="81" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A81" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B81" s="19">
+        <v>46.454767726161229</v>
+      </c>
+      <c r="C81" s="19">
+        <v>5.5154976968149203</v>
+      </c>
+      <c r="D81" s="26">
+        <v>3.0339999999999998</v>
+      </c>
+      <c r="E81" s="6"/>
+      <c r="F81" s="6"/>
+      <c r="G81" s="5">
+        <v>0.46894675925925927</v>
+      </c>
+    </row>
+    <row r="82" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A82" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B82" s="19">
+        <v>42.016806722689026</v>
+      </c>
+      <c r="C82" s="19"/>
+      <c r="D82" s="26">
+        <v>3.0539999999999998</v>
+      </c>
+      <c r="E82" s="6"/>
+      <c r="F82" s="6"/>
+      <c r="G82" s="5">
+        <v>0.4689814814814815</v>
+      </c>
+    </row>
+    <row r="83" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A83" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B83" s="19">
+        <v>43.243243243243327</v>
+      </c>
+      <c r="C83" s="19">
+        <v>3.9275319064876912</v>
+      </c>
+      <c r="D83" s="26">
+        <v>2.4729999999999999</v>
+      </c>
+      <c r="E83" s="6"/>
+      <c r="F83" s="6"/>
+      <c r="G83" s="5">
+        <v>0.46901620370370373</v>
+      </c>
+    </row>
+    <row r="84" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A84" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B84" s="19">
+        <v>144.48979591836752</v>
+      </c>
+      <c r="C84" s="19"/>
+      <c r="D84" s="26">
+        <v>2.6160000000000001</v>
+      </c>
+      <c r="E84" s="6"/>
+      <c r="F84" s="6"/>
+      <c r="G84" s="5">
+        <v>0.4690509259259259</v>
+      </c>
+    </row>
+    <row r="85" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A85" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B85" s="19">
+        <v>240.01979544704733</v>
+      </c>
+      <c r="C85" s="19">
+        <v>15.122709800124632</v>
+      </c>
+      <c r="D85" s="26">
+        <v>3.1349999999999998</v>
+      </c>
+      <c r="E85" s="6"/>
+      <c r="F85" s="6"/>
+      <c r="G85" s="5">
+        <v>0.46908564814814818</v>
+      </c>
+    </row>
+    <row r="86" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A86" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B86" s="19">
+        <v>191.19209085709622</v>
+      </c>
+      <c r="C86" s="19"/>
+      <c r="D86" s="26">
+        <v>2.9359999999999999</v>
+      </c>
+      <c r="E86" s="6"/>
+      <c r="F86" s="6"/>
+      <c r="G86" s="5">
+        <v>0.46912037037037035</v>
+      </c>
+    </row>
+    <row r="87" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A87" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B87" s="19">
+        <v>164.10842586544723</v>
+      </c>
+      <c r="C87" s="19">
+        <v>17.196570691909024</v>
+      </c>
+      <c r="D87" s="26">
+        <v>2.9329999999999998</v>
+      </c>
+      <c r="E87" s="6"/>
+      <c r="F87" s="6"/>
+      <c r="G87" s="5">
+        <v>0.46915509259259264</v>
+      </c>
+    </row>
+    <row r="88" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A88" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B88" s="19">
+        <v>119.19751531939913</v>
+      </c>
+      <c r="C88" s="19">
+        <v>9.506040177851494</v>
+      </c>
+      <c r="D88" s="26">
+        <v>2.6339999999999999</v>
+      </c>
+      <c r="E88" s="6"/>
+      <c r="F88" s="6"/>
+      <c r="G88" s="5">
+        <v>0.46918981481481481</v>
+      </c>
+    </row>
+    <row r="89" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A89" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B89" s="19">
+        <v>96.298777424216894</v>
+      </c>
+      <c r="C89" s="19">
+        <v>6.3675166712568405</v>
+      </c>
+      <c r="D89" s="26">
+        <v>2.97</v>
+      </c>
+      <c r="E89" s="6"/>
+      <c r="F89" s="6"/>
+      <c r="G89" s="5">
+        <v>0.46925925925925926</v>
+      </c>
+    </row>
+    <row r="90" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A90" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B90" s="19">
+        <v>96.842105263158203</v>
+      </c>
+      <c r="C90" s="19"/>
+      <c r="D90" s="26">
+        <v>2.4969999999999999</v>
+      </c>
+      <c r="E90" s="6"/>
+      <c r="F90" s="6"/>
+      <c r="G90" s="5">
+        <v>0.46929398148148144</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>